<commit_message>
Actualización automática desde SharePoint
</commit_message>
<xml_diff>
--- a/Base_Dato_Indisponibilidad_GEN_CL.xlsx
+++ b/Base_Dato_Indisponibilidad_GEN_CL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://engie.sharepoint.com/sites/OperacionesCentralMejillones-Administracin/Shared Documents/Administración/0.- Gerencia/02.- Operación/05.- EFOF_GEN_CL/05.- PRO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1361" documentId="8_{55EF2082-D0B7-4F26-90F5-434FA2717943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81B180EB-BEC6-40C2-A9D3-BE0EC3669F23}"/>
+  <xr:revisionPtr revIDLastSave="1363" documentId="8_{55EF2082-D0B7-4F26-90F5-434FA2717943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54B81C01-2C53-4623-BD08-7E66D7F8F3C5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{E052323F-F4D0-446A-B69C-8F538CB3C6F5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E052323F-F4D0-446A-B69C-8F538CB3C6F5}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DATOS_EVENTOS_GEN_CHILE" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <definedName name="SegmentaciónDeDatos_Sitio">#N/A</definedName>
     <definedName name="SegmentaciónDeDatos_Unidad">#N/A</definedName>
   </definedNames>
-  <calcPr calcId="191028" calcCompleted="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="125">
   <si>
     <t>ID</t>
   </si>
@@ -472,7 +472,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -513,11 +513,24 @@
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -548,16 +561,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="27" formatCode="dd/mm/yyyy\ h:mm"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -850,23 +853,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF87FAA9-1AA2-4036-9224-EC7F4966CB13}" name="BD_GEN_CL" displayName="BD_GEN_CL" ref="A10:J348" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A10:J348" xr:uid="{BF87FAA9-1AA2-4036-9224-EC7F4966CB13}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF87FAA9-1AA2-4036-9224-EC7F4966CB13}" name="BD_GEN_CL" displayName="BD_GEN_CL" ref="A10:J349" totalsRowShown="0" headerRowDxfId="11">
+  <autoFilter ref="A10:J349" xr:uid="{BF87FAA9-1AA2-4036-9224-EC7F4966CB13}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A11:I308">
     <sortCondition ref="F10:F308"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="3" xr3:uid="{AFE823F6-980E-4E32-B4F4-6ECDE10F377D}" name="ID"/>
-    <tableColumn id="1" xr3:uid="{CD000998-6E2C-4963-8605-37081D9C1A64}" name="Unidad" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{542F6635-555D-4F04-8C27-263AF6E0C9F1}" name="Sitio" dataDxfId="6">
+    <tableColumn id="1" xr3:uid="{CD000998-6E2C-4963-8605-37081D9C1A64}" name="Unidad" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{542F6635-555D-4F04-8C27-263AF6E0C9F1}" name="Sitio" dataDxfId="9">
       <calculatedColumnFormula>IF(OR(BD_GEN_CL[[#This Row],[Unidad]]="CTM3",BD_GEN_CL[[#This Row],[Unidad]]="CTA",BD_GEN_CL[[#This Row],[Unidad]]="CTH",BD_GEN_CL[[#This Row],[Unidad]]="IEM",BD_GEN_CL[[#This Row],[Unidad]]="CTM1",BD_GEN_CL[[#This Row],[Unidad]]="CTM2"),"CEM","CET")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{6D2AC534-BC70-4E36-815D-053C7EC9A0CE}" name="Carga_Disponible" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{FBB18F6C-27E4-42D9-9835-9152B6D0D871}" name="Estado_Op" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{21A32989-F167-49C0-9D41-2BD3A8923998}" name="Fecha_Hora_Inicio" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{713F74B7-95D9-4F96-AA1E-57E68B8A7FE7}" name="Fecha_Hora_Final" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{20481209-2CB3-4DCC-A330-D866983AA4F9}" name="Motivo" dataDxfId="1"/>
-    <tableColumn id="12" xr3:uid="{55FF6738-9798-4086-9AA1-DC8A3EF8081F}" name="Detalle" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{6D2AC534-BC70-4E36-815D-053C7EC9A0CE}" name="Carga_Disponible" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{FBB18F6C-27E4-42D9-9835-9152B6D0D871}" name="Estado_Op" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{21A32989-F167-49C0-9D41-2BD3A8923998}" name="Fecha_Hora_Inicio" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{713F74B7-95D9-4F96-AA1E-57E68B8A7FE7}" name="Fecha_Hora_Final" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{20481209-2CB3-4DCC-A330-D866983AA4F9}" name="Motivo" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{55FF6738-9798-4086-9AA1-DC8A3EF8081F}" name="Detalle" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{C2DE1A32-EBAC-4C95-A60E-FB6BAE643966}" name="Verificación"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -894,9 +897,9 @@
   </sortState>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{1EEE0FFC-B699-4850-9A13-72CF6FB78CA6}" name="Unidad"/>
-    <tableColumn id="2" xr3:uid="{BDB3B76C-8D9D-4A32-9C94-204172B9E68C}" name="Fecha_Hora_Inicio" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{A21A7F07-F50E-4006-B601-758B5E8BD7BE}" name="Fecha_Hora_Fin" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{F49EC928-7A7A-47BB-9275-EDE8B8DF6BC7}" name="Días_de_Mantenimiento" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{BDB3B76C-8D9D-4A32-9C94-204172B9E68C}" name="Fecha_Hora_Inicio" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{A21A7F07-F50E-4006-B601-758B5E8BD7BE}" name="Fecha_Hora_Fin" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{F49EC928-7A7A-47BB-9275-EDE8B8DF6BC7}" name="Días_de_Mantenimiento" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{E5C19B72-F1F0-4F1D-9466-99048BCEFC0C}" name="Motivo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1232,7 +1235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE341A5-48DC-491A-A7A3-9CB9E0074F67}">
-  <dimension ref="A9:J348"/>
+  <dimension ref="A9:J349"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -1251,7 +1254,7 @@
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <f>SUBTOTAL(103,BD_GEN_CL[Unidad])</f>
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -10514,6 +10517,24 @@
       <c r="J348" s="1" t="s">
         <v>23</v>
       </c>
+    </row>
+    <row r="349" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A349">
+        <v>339</v>
+      </c>
+      <c r="B349" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C349" s="16" t="str">
+        <f>IF(OR(BD_GEN_CL[[#This Row],[Unidad]]="CTM3",BD_GEN_CL[[#This Row],[Unidad]]="CTA",BD_GEN_CL[[#This Row],[Unidad]]="CTH",BD_GEN_CL[[#This Row],[Unidad]]="IEM",BD_GEN_CL[[#This Row],[Unidad]]="CTM1",BD_GEN_CL[[#This Row],[Unidad]]="CTM2"),"CEM","CET")</f>
+        <v>CET</v>
+      </c>
+      <c r="D349" s="14"/>
+      <c r="E349" s="13"/>
+      <c r="F349" s="15"/>
+      <c r="G349" s="15"/>
+      <c r="H349" s="11"/>
+      <c r="I349" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11017,6 +11038,29 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="33ab045e-9213-4eea-a9f2-a5b809105d1e">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100FB7AAE8C8816FD47B559A0CCF555AFF0" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5c9910934a78ddf693a6b708b52e9b37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f95d585e-e7a7-414c-955d-38a47c8579bd" xmlns:ns3="33ab045e-9213-4eea-a9f2-a5b809105d1e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a9c61c95b4e11caed4e46447c2ca01e7" ns2:_="" ns3:_="">
     <xsd:import namespace="f95d585e-e7a7-414c-955d-38a47c8579bd"/>
@@ -11219,30 +11263,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="33ab045e-9213-4eea-a9f2-a5b809105d1e">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59A15667-1AA5-4404-9771-E51F1A78CCAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3DCBC87-226F-4D83-ADFE-2178829A4AE4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="33ab045e-9213-4eea-a9f2-a5b809105d1e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A8D88B3-F603-4313-AC14-F1B2905698D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11261,24 +11300,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3DCBC87-226F-4D83-ADFE-2178829A4AE4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="33ab045e-9213-4eea-a9f2-a5b809105d1e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59A15667-1AA5-4404-9771-E51F1A78CCAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0a9b9e15-83d2-4075-9282-a04e05c6580a}" enabled="1" method="Standard" siteId="{24139d14-c62c-4c47-8bdd-ce71ea1d50cf}" contentBits="0" removed="0"/>

</xml_diff>